<commit_message>
add: suchtpozessHS26, change: letzte codechanges vom Ende letzten Semesters vor abgabe
</commit_message>
<xml_diff>
--- a/documentation/model_documentation/sections/scripts/results/forecast_v1/forecast_v1_summary.xlsx
+++ b/documentation/model_documentation/sections/scripts/results/forecast_v1/forecast_v1_summary.xlsx
@@ -17,10 +17,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="13">
   <si>
-    <t>time</t>
+    <t>Year</t>
   </si>
   <si>
-    <t>Year</t>
+    <t>Urban Land</t>
   </si>
   <si>
     <t>Aggricultural Land</t>
@@ -385,7 +385,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:13">
@@ -427,6 +427,252 @@
       </c>
       <c r="M1" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
+      <c r="A2">
+        <v>2025</v>
+      </c>
+      <c r="B2">
+        <v>181700</v>
+      </c>
+      <c r="C2">
+        <v>1600400</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>451800000</v>
+      </c>
+      <c r="G2">
+        <v>0.194633216695826</v>
+      </c>
+      <c r="H2">
+        <v>311491</v>
+      </c>
+      <c r="I2">
+        <v>1800000000</v>
+      </c>
+      <c r="J2">
+        <v>2.3</v>
+      </c>
+      <c r="K2">
+        <v>41650</v>
+      </c>
+      <c r="L2">
+        <v>0.47</v>
+      </c>
+      <c r="M2">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3">
+        <v>2030</v>
+      </c>
+      <c r="B3">
+        <v>191922.744452552</v>
+      </c>
+      <c r="C3">
+        <v>1590177.255547448</v>
+      </c>
+      <c r="D3">
+        <v>3698.470008324201</v>
+      </c>
+      <c r="E3">
+        <v>11095.4100249726</v>
+      </c>
+      <c r="F3">
+        <v>453200000</v>
+      </c>
+      <c r="G3">
+        <v>0.1860253465066438</v>
+      </c>
+      <c r="H3">
+        <v>295813.2749701979</v>
+      </c>
+      <c r="I3">
+        <v>1901270996.227813</v>
+      </c>
+      <c r="J3">
+        <v>2.251290893554687</v>
+      </c>
+      <c r="K3">
+        <v>43788.95937920093</v>
+      </c>
+      <c r="L3">
+        <v>0.47</v>
+      </c>
+      <c r="M3">
+        <v>29723.50214389793</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4">
+        <v>2035</v>
+      </c>
+      <c r="B4">
+        <v>211479.6972391221</v>
+      </c>
+      <c r="C4">
+        <v>1570620.302760878</v>
+      </c>
+      <c r="D4">
+        <v>4174.610699250789</v>
+      </c>
+      <c r="E4">
+        <v>12523.83209775237</v>
+      </c>
+      <c r="F4">
+        <v>452000000</v>
+      </c>
+      <c r="G4">
+        <v>0.1704718802986955</v>
+      </c>
+      <c r="H4">
+        <v>267746.5962469532</v>
+      </c>
+      <c r="I4">
+        <v>2095010759.661088</v>
+      </c>
+      <c r="J4">
+        <v>2.226307557616383</v>
+      </c>
+      <c r="K4">
+        <v>46134.65227191835</v>
+      </c>
+      <c r="L4">
+        <v>0.47</v>
+      </c>
+      <c r="M4">
+        <v>28220.9930777388</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5">
+        <v>2040</v>
+      </c>
+      <c r="B5">
+        <v>233032.4162546055</v>
+      </c>
+      <c r="C5">
+        <v>1549067.583745394</v>
+      </c>
+      <c r="D5">
+        <v>4568.530702382694</v>
+      </c>
+      <c r="E5">
+        <v>13705.59210714808</v>
+      </c>
+      <c r="F5">
+        <v>450000000</v>
+      </c>
+      <c r="G5">
+        <v>0.1561636723531312</v>
+      </c>
+      <c r="H5">
+        <v>241908.0826008724</v>
+      </c>
+      <c r="I5">
+        <v>2308521459.86951</v>
+      </c>
+      <c r="J5">
+        <v>2.213493381373857</v>
+      </c>
+      <c r="K5">
+        <v>48741.18507130406</v>
+      </c>
+      <c r="L5">
+        <v>0.47</v>
+      </c>
+      <c r="M5">
+        <v>26175.68624959282</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6">
+        <v>2045</v>
+      </c>
+      <c r="B6">
+        <v>256910.6413297726</v>
+      </c>
+      <c r="C6">
+        <v>1525189.358670227</v>
+      </c>
+      <c r="D6">
+        <v>5146.767929568935</v>
+      </c>
+      <c r="E6">
+        <v>15440.30378870681</v>
+      </c>
+      <c r="F6">
+        <v>447500000</v>
+      </c>
+      <c r="G6">
+        <v>0.143067630231099</v>
+      </c>
+      <c r="H6">
+        <v>218205.2271986391</v>
+      </c>
+      <c r="I6">
+        <v>2545069644.43363</v>
+      </c>
+      <c r="J6">
+        <v>2.206920875877393</v>
+      </c>
+      <c r="K6">
+        <v>51652.21825278555</v>
+      </c>
+      <c r="L6">
+        <v>0.47</v>
+      </c>
+      <c r="M6">
+        <v>24088.17548004497</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7">
+        <v>2050</v>
+      </c>
+      <c r="B7">
+        <v>284234.3731317717</v>
+      </c>
+      <c r="C7">
+        <v>1497865.626868228</v>
+      </c>
+      <c r="D7">
+        <v>5993.509827161247</v>
+      </c>
+      <c r="E7">
+        <v>17980.52948148374</v>
+      </c>
+      <c r="F7">
+        <v>445000000</v>
+      </c>
+      <c r="G7">
+        <v>0.1309377165788006</v>
+      </c>
+      <c r="H7">
+        <v>196127.1049239996</v>
+      </c>
+      <c r="I7">
+        <v>2815750531.850242</v>
+      </c>
+      <c r="J7">
+        <v>2.203549779079326</v>
+      </c>
+      <c r="K7">
+        <v>54924.57968106154</v>
+      </c>
+      <c r="L7">
+        <v>0.47</v>
+      </c>
+      <c r="M7">
+        <v>22099.19778561492</v>
       </c>
     </row>
   </sheetData>

</xml_diff>